<commit_message>
feat(backend): Precess sidereal coordinates, improve determination of rising targets, program edits and related ephemeris updates, resource updates, support for new GPP inst
</commit_message>
<xml_diff>
--- a/backend/scheduler/services/resource/data/validation/telescope_schedules.xlsx
+++ b/backend/scheduler/services/resource/data/validation/telescope_schedules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sergio.troncoso/PycharmProjects/scheduler/scheduler/services/resource/data/validation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bmiller/python/scheduler/backend/scheduler/services/resource/data/validation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB68D29-82FC-4C49-A6F8-A5F2E0F30DF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E7A96A4-7EC2-1A46-B0A3-0DEC1C93487D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19400" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GS" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24007" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24007" uniqueCount="88">
   <si>
     <t>Local Date</t>
   </si>
@@ -282,6 +282,9 @@
   </si>
   <si>
     <t>Queue | Visitor: `Alopeke</t>
+  </si>
+  <si>
+    <t>Classical: GS-2014B-C-500, GS-2014B-C-502</t>
   </si>
 </sst>
 </file>
@@ -14649,7 +14652,7 @@
         <v>25</v>
       </c>
       <c r="C189" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D189" s="1" t="s">
         <v>27</v>
@@ -14724,7 +14727,7 @@
         <v>25</v>
       </c>
       <c r="C190" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D190" s="1" t="s">
         <v>27</v>
@@ -14799,7 +14802,7 @@
         <v>25</v>
       </c>
       <c r="C191" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D191" s="1" t="s">
         <v>27</v>
@@ -14874,7 +14877,7 @@
         <v>25</v>
       </c>
       <c r="C192" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D192" s="1" t="s">
         <v>27</v>
@@ -14949,7 +14952,7 @@
         <v>25</v>
       </c>
       <c r="C193" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D193" s="1" t="s">
         <v>27</v>
@@ -15024,7 +15027,7 @@
         <v>25</v>
       </c>
       <c r="C194" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D194" s="1" t="s">
         <v>27</v>
@@ -15099,7 +15102,7 @@
         <v>25</v>
       </c>
       <c r="C195" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D195" s="1" t="s">
         <v>27</v>
@@ -17697,7 +17700,7 @@
         <v>25</v>
       </c>
       <c r="C232" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D232" s="1" t="s">
         <v>27</v>
@@ -17772,7 +17775,7 @@
         <v>25</v>
       </c>
       <c r="C233" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D233" s="1" t="s">
         <v>27</v>
@@ -17847,7 +17850,7 @@
         <v>25</v>
       </c>
       <c r="C234" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D234" s="1" t="s">
         <v>27</v>
@@ -17922,7 +17925,7 @@
         <v>25</v>
       </c>
       <c r="C235" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D235" s="1" t="s">
         <v>27</v>
@@ -17997,7 +18000,7 @@
         <v>25</v>
       </c>
       <c r="C236" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D236" s="1" t="s">
         <v>27</v>
@@ -22122,7 +22125,7 @@
         <v>25</v>
       </c>
       <c r="C291" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D291" s="1" t="s">
         <v>27</v>
@@ -22197,7 +22200,7 @@
         <v>25</v>
       </c>
       <c r="C292" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D292" s="1" t="s">
         <v>27</v>
@@ -22272,7 +22275,7 @@
         <v>25</v>
       </c>
       <c r="C293" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D293" s="1" t="s">
         <v>27</v>
@@ -22347,7 +22350,7 @@
         <v>25</v>
       </c>
       <c r="C294" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D294" s="1" t="s">
         <v>27</v>
@@ -22422,7 +22425,7 @@
         <v>25</v>
       </c>
       <c r="C295" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D295" s="1" t="s">
         <v>27</v>
@@ -24510,7 +24513,7 @@
         <v>25</v>
       </c>
       <c r="C323" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D323" s="1" t="s">
         <v>27</v>
@@ -24585,7 +24588,7 @@
         <v>25</v>
       </c>
       <c r="C324" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D324" s="1" t="s">
         <v>27</v>
@@ -24660,7 +24663,7 @@
         <v>25</v>
       </c>
       <c r="C325" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D325" s="1" t="s">
         <v>27</v>
@@ -24735,7 +24738,7 @@
         <v>25</v>
       </c>
       <c r="C326" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D326" s="1" t="s">
         <v>27</v>
@@ -24810,7 +24813,7 @@
         <v>25</v>
       </c>
       <c r="C327" s="1" t="s">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="D327" s="1" t="s">
         <v>27</v>

</xml_diff>